<commit_message>
updated balde and producao - base 12/03/2026
</commit_message>
<xml_diff>
--- a/first-atlas/producao_2026-03.xlsx
+++ b/first-atlas/producao_2026-03.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\augustoalmeida\Augusto\bots_comissionamento\bot_atlas\first-atlas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3EA949C-1415-45F1-9CA3-816AFB1C06B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C4B4DA-6239-449B-8558-F43A5DFB9D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F5572131-3C84-4D9C-B555-72DCC3B1940B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3510" uniqueCount="1068">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3584" uniqueCount="1096">
   <si>
     <t>DATA_BASE</t>
   </si>
@@ -3243,6 +3243,90 @@
   </si>
   <si>
     <t>BKO</t>
+  </si>
+  <si>
+    <t>06029505000165</t>
+  </si>
+  <si>
+    <t>NEW DREAMS COMERCIO E SERVICOS DE INFORMATICA LTDA</t>
+  </si>
+  <si>
+    <t>19344602000194</t>
+  </si>
+  <si>
+    <t>PGA SOLUCOES TECNICAS LTDA</t>
+  </si>
+  <si>
+    <t>09324631000130</t>
+  </si>
+  <si>
+    <t>ESTRELA AZUL COMERCIO DE CEREAIS LTDA</t>
+  </si>
+  <si>
+    <t>11659063000170</t>
+  </si>
+  <si>
+    <t>GREGOLINI VEICULOS LTDA</t>
+  </si>
+  <si>
+    <t>64847157000130</t>
+  </si>
+  <si>
+    <t>DN REPARO GERAL LTDA</t>
+  </si>
+  <si>
+    <t>17840308000148</t>
+  </si>
+  <si>
+    <t>MP MOVEIS PROJETADOS LTDA</t>
+  </si>
+  <si>
+    <t>63308182000182</t>
+  </si>
+  <si>
+    <t>MV SERVICOS DE MOTO LTDA</t>
+  </si>
+  <si>
+    <t>62406655000111</t>
+  </si>
+  <si>
+    <t>GTPD ALIMENTACAO LTDA</t>
+  </si>
+  <si>
+    <t>59428502000160</t>
+  </si>
+  <si>
+    <t>TABACARIA FENIX LTDA</t>
+  </si>
+  <si>
+    <t>60103323000132</t>
+  </si>
+  <si>
+    <t>ENERGIZAR SOLUCOES ELETRICAS LTDA</t>
+  </si>
+  <si>
+    <t>65372525000101</t>
+  </si>
+  <si>
+    <t>PRIME SOLUTIONS GROUP LTDA</t>
+  </si>
+  <si>
+    <t>65097911000124</t>
+  </si>
+  <si>
+    <t>CLAODECIR LODI RISSINI CLAODECIR LODI RISSINI</t>
+  </si>
+  <si>
+    <t>50867370000107</t>
+  </si>
+  <si>
+    <t>GUSTAVO LIMA BATISTA</t>
+  </si>
+  <si>
+    <t>62187027000192</t>
+  </si>
+  <si>
+    <t>ALBA CRISTINA BATISTA</t>
   </si>
 </sst>
 </file>
@@ -3615,12 +3699,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A45A88-3D17-4433-986A-11075963C36F}">
-  <dimension ref="A1:I503"/>
+  <dimension ref="A1:I517"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11849,11 +11934,11 @@
       <c r="C287" t="s">
         <v>622</v>
       </c>
-      <c r="D287" t="s">
-        <v>1061</v>
-      </c>
-      <c r="E287" t="s">
-        <v>1062</v>
+      <c r="D287" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E287" t="e">
+        <v>#N/A</v>
       </c>
       <c r="F287" t="s">
         <v>17</v>
@@ -13268,7 +13353,7 @@
         <v>8</v>
       </c>
       <c r="H336" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I336">
         <v>0</v>
@@ -13674,7 +13759,7 @@
         <v>8</v>
       </c>
       <c r="H350" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I350">
         <v>0</v>
@@ -14370,7 +14455,7 @@
         <v>31</v>
       </c>
       <c r="H374" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I374">
         <v>0</v>
@@ -14428,7 +14513,7 @@
         <v>8</v>
       </c>
       <c r="H376" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I376">
         <v>0</v>
@@ -14515,7 +14600,7 @@
         <v>8</v>
       </c>
       <c r="H379" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I379">
         <v>0</v>
@@ -14950,7 +15035,7 @@
         <v>31</v>
       </c>
       <c r="H394" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I394">
         <v>0</v>
@@ -15008,7 +15093,7 @@
         <v>8</v>
       </c>
       <c r="H396" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I396">
         <v>0</v>
@@ -15414,7 +15499,7 @@
         <v>8</v>
       </c>
       <c r="H410" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I410">
         <v>0</v>
@@ -15588,10 +15673,13 @@
         <v>8</v>
       </c>
       <c r="H416" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="417" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I416">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="417" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A417" s="1">
         <v>46092</v>
       </c>
@@ -15616,8 +15704,11 @@
       <c r="H417" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="418" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I417">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="418" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A418" s="1">
         <v>46092</v>
       </c>
@@ -15642,8 +15733,11 @@
       <c r="H418" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="419" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I418">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A419" s="1">
         <v>46092</v>
       </c>
@@ -15668,8 +15762,11 @@
       <c r="H419" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="420" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I419">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A420" s="1">
         <v>46092</v>
       </c>
@@ -15694,8 +15791,11 @@
       <c r="H420" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="421" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I420">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A421" s="1">
         <v>46092</v>
       </c>
@@ -15718,10 +15818,13 @@
         <v>8</v>
       </c>
       <c r="H421" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="422" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I421">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="422" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A422" s="1">
         <v>46092</v>
       </c>
@@ -15746,8 +15849,11 @@
       <c r="H422" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="423" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I422">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="423" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A423" s="1">
         <v>46092</v>
       </c>
@@ -15772,8 +15878,11 @@
       <c r="H423" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="424" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I423">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="424" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A424" s="1">
         <v>46092</v>
       </c>
@@ -15798,8 +15907,11 @@
       <c r="H424" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="425" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I424">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A425" s="1">
         <v>46092</v>
       </c>
@@ -15824,8 +15936,11 @@
       <c r="H425" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="426" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I425">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="426" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A426" s="1">
         <v>46092</v>
       </c>
@@ -15850,8 +15965,11 @@
       <c r="H426" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="427" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I426">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A427" s="1">
         <v>46092</v>
       </c>
@@ -15874,10 +15992,13 @@
         <v>8</v>
       </c>
       <c r="H427" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="428" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I427">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A428" s="1">
         <v>46092</v>
       </c>
@@ -15900,10 +16021,13 @@
         <v>8</v>
       </c>
       <c r="H428" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="429" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I428">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A429" s="1">
         <v>46092</v>
       </c>
@@ -15926,10 +16050,13 @@
         <v>7</v>
       </c>
       <c r="H429" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="430" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I429" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="430" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A430" s="1">
         <v>46092</v>
       </c>
@@ -15954,8 +16081,11 @@
       <c r="H430" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="431" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I430">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="431" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A431" s="1">
         <v>46092</v>
       </c>
@@ -15980,8 +16110,11 @@
       <c r="H431" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="432" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I431">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="432" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A432" s="1">
         <v>46092</v>
       </c>
@@ -16006,8 +16139,11 @@
       <c r="H432" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="433" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I432">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A433" s="1">
         <v>46092</v>
       </c>
@@ -16032,8 +16168,11 @@
       <c r="H433" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="434" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I433">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A434" s="1">
         <v>46092</v>
       </c>
@@ -16058,8 +16197,11 @@
       <c r="H434" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="435" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I434">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A435" s="1">
         <v>46092</v>
       </c>
@@ -16084,8 +16226,11 @@
       <c r="H435" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="436" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I435">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="436" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A436" s="1">
         <v>46092</v>
       </c>
@@ -16110,8 +16255,11 @@
       <c r="H436" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="437" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I436">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A437" s="1">
         <v>46092</v>
       </c>
@@ -16136,8 +16284,11 @@
       <c r="H437" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="438" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I437">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="438" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A438" s="1">
         <v>46092</v>
       </c>
@@ -16162,8 +16313,11 @@
       <c r="H438" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="439" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I438">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="439" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A439" s="1">
         <v>46092</v>
       </c>
@@ -16188,8 +16342,11 @@
       <c r="H439" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="440" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I439">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="440" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A440" s="1">
         <v>46092</v>
       </c>
@@ -16212,10 +16369,13 @@
         <v>8</v>
       </c>
       <c r="H440" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="441" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I440">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="441" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A441" s="1">
         <v>46092</v>
       </c>
@@ -16240,8 +16400,11 @@
       <c r="H441" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="442" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I441">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="442" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A442" s="1">
         <v>46092</v>
       </c>
@@ -16264,10 +16427,13 @@
         <v>934</v>
       </c>
       <c r="H442" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="443" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I442">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="443" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A443" s="1">
         <v>46092</v>
       </c>
@@ -16290,10 +16456,13 @@
         <v>8</v>
       </c>
       <c r="H443" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="444" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I443">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="444" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A444" s="1">
         <v>46092</v>
       </c>
@@ -16316,10 +16485,13 @@
         <v>8</v>
       </c>
       <c r="H444" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="445" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I444">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="445" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A445" s="1">
         <v>46092</v>
       </c>
@@ -16344,8 +16516,11 @@
       <c r="H445" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="446" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I445">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="446" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A446" s="1">
         <v>46092</v>
       </c>
@@ -16368,10 +16543,13 @@
         <v>8</v>
       </c>
       <c r="H446" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="447" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I446">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="447" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A447" s="1">
         <v>46092</v>
       </c>
@@ -16396,8 +16574,11 @@
       <c r="H447" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="448" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I447">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="448" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A448" s="1">
         <v>46092</v>
       </c>
@@ -16422,8 +16603,11 @@
       <c r="H448" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="449" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I448">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="449" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A449" s="1">
         <v>46092</v>
       </c>
@@ -16448,8 +16632,11 @@
       <c r="H449" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="450" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I449">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="450" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A450" s="1">
         <v>46092</v>
       </c>
@@ -16472,10 +16659,13 @@
         <v>934</v>
       </c>
       <c r="H450" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="451" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I450">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="451" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A451" s="1">
         <v>46092</v>
       </c>
@@ -16500,8 +16690,11 @@
       <c r="H451" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="452" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I451">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="452" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A452" s="1">
         <v>46092</v>
       </c>
@@ -16526,8 +16719,11 @@
       <c r="H452" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="453" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I452">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="453" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A453" s="1">
         <v>46092</v>
       </c>
@@ -16550,10 +16746,10 @@
         <v>13</v>
       </c>
       <c r="H453" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="454" spans="1:8" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="454" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A454" s="1">
         <v>46092</v>
       </c>
@@ -16578,8 +16774,11 @@
       <c r="H454" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="455" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I454">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="455" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A455" s="1">
         <v>46092</v>
       </c>
@@ -16604,8 +16803,11 @@
       <c r="H455" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="456" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I455">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="456" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A456" s="1">
         <v>46092</v>
       </c>
@@ -16628,10 +16830,13 @@
         <v>8</v>
       </c>
       <c r="H456" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="457" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I456">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A457" s="1">
         <v>46092</v>
       </c>
@@ -16656,8 +16861,11 @@
       <c r="H457" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="458" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I457">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="458" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A458" s="1">
         <v>46092</v>
       </c>
@@ -16682,8 +16890,11 @@
       <c r="H458" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="459" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I458">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="459" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A459" s="1">
         <v>46092</v>
       </c>
@@ -16708,8 +16919,11 @@
       <c r="H459" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="460" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I459">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="460" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A460" s="1">
         <v>46092</v>
       </c>
@@ -16734,8 +16948,11 @@
       <c r="H460" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="461" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I460">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="461" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A461" s="1">
         <v>46092</v>
       </c>
@@ -16760,8 +16977,11 @@
       <c r="H461" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="462" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I461">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="462" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A462" s="1">
         <v>46092</v>
       </c>
@@ -16784,10 +17004,13 @@
         <v>8</v>
       </c>
       <c r="H462" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="463" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I462" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="463" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A463" s="1">
         <v>46092</v>
       </c>
@@ -16812,8 +17035,11 @@
       <c r="H463" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="464" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I463">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="464" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A464" s="1">
         <v>46092</v>
       </c>
@@ -16838,8 +17064,11 @@
       <c r="H464" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="465" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I464">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="465" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A465" s="1">
         <v>46092</v>
       </c>
@@ -16864,8 +17093,11 @@
       <c r="H465" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="466" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I465">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A466" s="1">
         <v>46092</v>
       </c>
@@ -16890,8 +17122,11 @@
       <c r="H466" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="467" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I466">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="467" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A467" s="1">
         <v>46092</v>
       </c>
@@ -16914,10 +17149,13 @@
         <v>8</v>
       </c>
       <c r="H467" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="468" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I467" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="468" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A468" s="1">
         <v>46092</v>
       </c>
@@ -16942,8 +17180,11 @@
       <c r="H468" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="469" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I468">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="469" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A469" s="1">
         <v>46092</v>
       </c>
@@ -16968,8 +17209,11 @@
       <c r="H469" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="470" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I469">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A470" s="1">
         <v>46092</v>
       </c>
@@ -16992,10 +17236,13 @@
         <v>8</v>
       </c>
       <c r="H470" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="471" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I470">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="471" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A471" s="1">
         <v>46092</v>
       </c>
@@ -17020,8 +17267,11 @@
       <c r="H471" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="472" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I471">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="472" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A472" s="1">
         <v>46092</v>
       </c>
@@ -17044,10 +17294,13 @@
         <v>8</v>
       </c>
       <c r="H472" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="473" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I472">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="473" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A473" s="1">
         <v>46092</v>
       </c>
@@ -17070,10 +17323,13 @@
         <v>8</v>
       </c>
       <c r="H473" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="474" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I473">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="474" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A474" s="1">
         <v>46092</v>
       </c>
@@ -17098,8 +17354,11 @@
       <c r="H474" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="475" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I474">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="475" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A475" s="1">
         <v>46092</v>
       </c>
@@ -17122,10 +17381,13 @@
         <v>8</v>
       </c>
       <c r="H475" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="476" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I475" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="476" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A476" s="1">
         <v>46092</v>
       </c>
@@ -17148,10 +17410,13 @@
         <v>635</v>
       </c>
       <c r="H476" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="477" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I476">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A477" s="1">
         <v>46092</v>
       </c>
@@ -17174,10 +17439,13 @@
         <v>10</v>
       </c>
       <c r="H477" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="478" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I477">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A478" s="1">
         <v>46092</v>
       </c>
@@ -17202,8 +17470,11 @@
       <c r="H478" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="479" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I478">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A479" s="1">
         <v>46092</v>
       </c>
@@ -17228,8 +17499,11 @@
       <c r="H479" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="480" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I479">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="480" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A480" s="1">
         <v>46092</v>
       </c>
@@ -17254,8 +17528,11 @@
       <c r="H480" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="481" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I480">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A481" s="1">
         <v>46092</v>
       </c>
@@ -17278,10 +17555,13 @@
         <v>8</v>
       </c>
       <c r="H481" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="482" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I481">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="482" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A482" s="1">
         <v>46092</v>
       </c>
@@ -17304,10 +17584,13 @@
         <v>8</v>
       </c>
       <c r="H482" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="483" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I482">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="483" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A483" s="1">
         <v>46092</v>
       </c>
@@ -17332,8 +17615,11 @@
       <c r="H483" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="484" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I483">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="484" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A484" s="1">
         <v>46092</v>
       </c>
@@ -17358,8 +17644,11 @@
       <c r="H484" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="485" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I484">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="485" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A485" s="1">
         <v>46092</v>
       </c>
@@ -17382,10 +17671,13 @@
         <v>8</v>
       </c>
       <c r="H485" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="486" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I485" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="486" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A486" s="1">
         <v>46092</v>
       </c>
@@ -17410,8 +17702,11 @@
       <c r="H486" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="487" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I486">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="487" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A487" s="1">
         <v>46092</v>
       </c>
@@ -17434,10 +17729,13 @@
         <v>8</v>
       </c>
       <c r="H487" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="488" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I487" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="488" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A488" s="1">
         <v>46092</v>
       </c>
@@ -17462,8 +17760,11 @@
       <c r="H488" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="489" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I488">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="489" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A489" s="1">
         <v>46092</v>
       </c>
@@ -17488,8 +17789,11 @@
       <c r="H489" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="490" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I489">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="490" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A490" s="1">
         <v>46092</v>
       </c>
@@ -17512,10 +17816,13 @@
         <v>8</v>
       </c>
       <c r="H490" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="491" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I490">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="491" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A491" s="1">
         <v>46092</v>
       </c>
@@ -17538,10 +17845,13 @@
         <v>8</v>
       </c>
       <c r="H491" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="492" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I491">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="492" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A492" s="1">
         <v>46092</v>
       </c>
@@ -17566,8 +17876,11 @@
       <c r="H492" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="493" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I492">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="493" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A493" s="1">
         <v>46092</v>
       </c>
@@ -17592,8 +17905,11 @@
       <c r="H493" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="494" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I493">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="494" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A494" s="1">
         <v>46092</v>
       </c>
@@ -17618,8 +17934,11 @@
       <c r="H494" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="495" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I494">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="495" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A495" s="1">
         <v>46092</v>
       </c>
@@ -17644,8 +17963,11 @@
       <c r="H495" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="496" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I495">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="496" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A496" s="1">
         <v>46092</v>
       </c>
@@ -17669,6 +17991,9 @@
       </c>
       <c r="H496" t="s">
         <v>21</v>
+      </c>
+      <c r="I496">
+        <v>0</v>
       </c>
     </row>
     <row r="497" spans="1:9" x14ac:dyDescent="0.25">
@@ -17854,6 +18179,319 @@
       </c>
       <c r="I503">
         <v>0</v>
+      </c>
+    </row>
+    <row r="504" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A504" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B504" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C504" t="s">
+        <v>1069</v>
+      </c>
+      <c r="F504" t="s">
+        <v>16</v>
+      </c>
+      <c r="G504" t="s">
+        <v>8</v>
+      </c>
+      <c r="H504" t="s">
+        <v>19</v>
+      </c>
+      <c r="I504">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="505" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A505" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B505" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C505" t="s">
+        <v>1071</v>
+      </c>
+      <c r="F505" t="s">
+        <v>20</v>
+      </c>
+      <c r="G505" t="s">
+        <v>8</v>
+      </c>
+      <c r="H505" t="s">
+        <v>19</v>
+      </c>
+      <c r="I505">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="506" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A506" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B506" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C506" t="s">
+        <v>1073</v>
+      </c>
+      <c r="F506" t="s">
+        <v>39</v>
+      </c>
+      <c r="G506" t="s">
+        <v>8</v>
+      </c>
+      <c r="H506" t="s">
+        <v>19</v>
+      </c>
+      <c r="I506">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="507" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A507" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B507" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C507" t="s">
+        <v>1075</v>
+      </c>
+      <c r="F507" t="s">
+        <v>39</v>
+      </c>
+      <c r="G507" t="s">
+        <v>8</v>
+      </c>
+      <c r="H507" t="s">
+        <v>19</v>
+      </c>
+      <c r="I507">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="508" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A508" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B508" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C508" t="s">
+        <v>1077</v>
+      </c>
+      <c r="F508" t="s">
+        <v>39</v>
+      </c>
+      <c r="G508" t="s">
+        <v>8</v>
+      </c>
+      <c r="H508" t="s">
+        <v>19</v>
+      </c>
+      <c r="I508">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="509" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A509" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B509" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C509" t="s">
+        <v>1079</v>
+      </c>
+      <c r="F509" t="s">
+        <v>20</v>
+      </c>
+      <c r="G509" t="s">
+        <v>8</v>
+      </c>
+      <c r="H509" t="s">
+        <v>19</v>
+      </c>
+      <c r="I509">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="510" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A510" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C510" t="s">
+        <v>1081</v>
+      </c>
+      <c r="F510" t="s">
+        <v>39</v>
+      </c>
+      <c r="G510" t="s">
+        <v>8</v>
+      </c>
+      <c r="H510" t="s">
+        <v>19</v>
+      </c>
+      <c r="I510">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="511" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A511" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B511" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C511" t="s">
+        <v>1083</v>
+      </c>
+      <c r="F511" t="s">
+        <v>39</v>
+      </c>
+      <c r="G511" t="s">
+        <v>8</v>
+      </c>
+      <c r="H511" t="s">
+        <v>19</v>
+      </c>
+      <c r="I511">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="512" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A512" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B512" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C512" t="s">
+        <v>1085</v>
+      </c>
+      <c r="F512" t="s">
+        <v>20</v>
+      </c>
+      <c r="G512" t="s">
+        <v>8</v>
+      </c>
+      <c r="H512" t="s">
+        <v>19</v>
+      </c>
+      <c r="I512">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="513" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A513" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B513" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C513" t="s">
+        <v>1087</v>
+      </c>
+      <c r="F513" t="s">
+        <v>39</v>
+      </c>
+      <c r="G513" t="s">
+        <v>8</v>
+      </c>
+      <c r="H513" t="s">
+        <v>19</v>
+      </c>
+      <c r="I513">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="514" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A514" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B514" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C514" t="s">
+        <v>1089</v>
+      </c>
+      <c r="F514" t="s">
+        <v>41</v>
+      </c>
+      <c r="G514" t="s">
+        <v>8</v>
+      </c>
+      <c r="H514" t="s">
+        <v>19</v>
+      </c>
+      <c r="I514">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="515" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A515" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B515" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C515" t="s">
+        <v>1091</v>
+      </c>
+      <c r="F515" t="s">
+        <v>39</v>
+      </c>
+      <c r="G515" t="s">
+        <v>40</v>
+      </c>
+      <c r="H515" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="516" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A516" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B516" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C516" t="s">
+        <v>1093</v>
+      </c>
+      <c r="F516" t="s">
+        <v>39</v>
+      </c>
+      <c r="G516" t="s">
+        <v>40</v>
+      </c>
+      <c r="H516" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="517" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A517" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B517" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C517" t="s">
+        <v>1095</v>
+      </c>
+      <c r="F517" t="s">
+        <v>39</v>
+      </c>
+      <c r="G517" t="s">
+        <v>40</v>
+      </c>
+      <c r="H517" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated and fixed producao
</commit_message>
<xml_diff>
--- a/first-atlas/producao_2026-03.xlsx
+++ b/first-atlas/producao_2026-03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\augustoalmeida\Augusto\bots_comissionamento\bot_atlas\first-atlas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E63B3B-0EC3-4415-8E09-0ACB01E0739A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0F4D4F-94D1-4416-BA6A-27874D0B80B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F5572131-3C84-4D9C-B555-72DCC3B1940B}"/>
+    <workbookView xWindow="-13620" yWindow="-3225" windowWidth="13740" windowHeight="21840" xr2:uid="{F5572131-3C84-4D9C-B555-72DCC3B1940B}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4827" uniqueCount="1451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4837" uniqueCount="1450">
   <si>
     <t>DATA_BASE</t>
   </si>
@@ -4377,9 +4377,6 @@
   </si>
   <si>
     <t>EMPORIO E DISTRIBUIDORA BOI DE OURO LTDA</t>
-  </si>
-  <si>
-    <t>LETICIA VIVIANE CARVALHO DA PENA</t>
   </si>
   <si>
     <t>62921625000143</t>
@@ -4434,58 +4431,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -11815,10 +11761,10 @@
         <v>10</v>
       </c>
       <c r="H246" t="s">
-        <v>29</v>
-      </c>
-      <c r="I246" t="s">
-        <v>34</v>
+        <v>23</v>
+      </c>
+      <c r="I246">
+        <v>0</v>
       </c>
     </row>
     <row r="247" spans="1:9" x14ac:dyDescent="0.25">
@@ -13427,7 +13373,7 @@
         <v>8</v>
       </c>
       <c r="H302" t="s">
-        <v>29</v>
+        <v>699</v>
       </c>
       <c r="I302">
         <v>0</v>
@@ -16660,7 +16606,7 @@
         <v>8</v>
       </c>
       <c r="H414" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="415" spans="1:9" x14ac:dyDescent="0.25">
@@ -21281,7 +21227,7 @@
         <v>8</v>
       </c>
       <c r="H575" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I575">
         <v>0</v>
@@ -21962,7 +21908,7 @@
         <v>7</v>
       </c>
       <c r="H599" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I599">
         <v>0</v>
@@ -21991,7 +21937,7 @@
         <v>7</v>
       </c>
       <c r="H600" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I600">
         <v>0</v>
@@ -22078,7 +22024,7 @@
         <v>7</v>
       </c>
       <c r="H603" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I603">
         <v>0</v>
@@ -22107,7 +22053,7 @@
         <v>8</v>
       </c>
       <c r="H604" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I604">
         <v>0</v>
@@ -22368,7 +22314,7 @@
         <v>7</v>
       </c>
       <c r="H613" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I613">
         <v>0</v>
@@ -22484,7 +22430,7 @@
         <v>7</v>
       </c>
       <c r="H617" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I617">
         <v>0</v>
@@ -22542,7 +22488,7 @@
         <v>8</v>
       </c>
       <c r="H619" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="I619">
         <v>0</v>
@@ -23116,7 +23062,7 @@
         <v>8</v>
       </c>
       <c r="H639" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I639">
         <v>0</v>
@@ -23174,7 +23120,7 @@
         <v>10</v>
       </c>
       <c r="H641" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I641">
         <v>0</v>
@@ -23348,7 +23294,7 @@
         <v>8</v>
       </c>
       <c r="H647" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I647">
         <v>0</v>
@@ -23632,7 +23578,7 @@
         <v>8</v>
       </c>
       <c r="H657" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I657">
         <v>0</v>
@@ -23661,7 +23607,7 @@
         <v>8</v>
       </c>
       <c r="H658" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I658">
         <v>0</v>
@@ -23912,6 +23858,9 @@
       <c r="H667" t="s">
         <v>19</v>
       </c>
+      <c r="I667">
+        <v>0</v>
+      </c>
     </row>
     <row r="668" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A668" s="1">
@@ -23935,6 +23884,9 @@
       <c r="H668" t="s">
         <v>19</v>
       </c>
+      <c r="I668">
+        <v>0</v>
+      </c>
     </row>
     <row r="669" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A669" s="1">
@@ -23958,6 +23910,9 @@
       <c r="H669" t="s">
         <v>19</v>
       </c>
+      <c r="I669">
+        <v>0</v>
+      </c>
     </row>
     <row r="670" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A670" s="1">
@@ -23981,6 +23936,9 @@
       <c r="H670" t="s">
         <v>19</v>
       </c>
+      <c r="I670">
+        <v>0</v>
+      </c>
     </row>
     <row r="671" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A671" s="1">
@@ -24004,6 +23962,9 @@
       <c r="H671" t="s">
         <v>19</v>
       </c>
+      <c r="I671">
+        <v>0</v>
+      </c>
     </row>
     <row r="672" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A672" s="1">
@@ -24027,8 +23988,11 @@
       <c r="H672" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="673" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I672">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A673" s="1">
         <v>46095</v>
       </c>
@@ -24053,8 +24017,11 @@
       <c r="H673" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="674" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I673">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A674" s="1">
         <v>46095</v>
       </c>
@@ -24079,8 +24046,11 @@
       <c r="H674" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="675" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I674">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="675" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A675" s="1">
         <v>46095</v>
       </c>
@@ -24103,10 +24073,13 @@
         <v>8</v>
       </c>
       <c r="H675" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="676" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I675">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="676" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A676" s="1">
         <v>46095</v>
       </c>
@@ -24132,7 +24105,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="677" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="677" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A677" s="1">
         <v>46095</v>
       </c>
@@ -24155,10 +24128,10 @@
         <v>8</v>
       </c>
       <c r="H677" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="678" spans="1:8" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="678" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A678" s="1">
         <v>46095</v>
       </c>
@@ -24181,10 +24154,13 @@
         <v>8</v>
       </c>
       <c r="H678" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="679" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I678">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="679" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A679" s="1">
         <v>46095</v>
       </c>
@@ -24209,8 +24185,11 @@
       <c r="H679" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="680" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I679">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="680" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A680" s="1">
         <v>46095</v>
       </c>
@@ -24235,8 +24214,11 @@
       <c r="H680" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="681" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I680">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A681" s="1">
         <v>46095</v>
       </c>
@@ -24261,8 +24243,11 @@
       <c r="H681" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="682" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I681">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="682" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A682" s="1">
         <v>46095</v>
       </c>
@@ -24284,8 +24269,11 @@
       <c r="H682" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="683" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I682">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="683" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A683" s="1">
         <v>46095</v>
       </c>
@@ -24310,8 +24298,11 @@
       <c r="H683" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="684" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I683">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="684" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A684" s="1">
         <v>46095</v>
       </c>
@@ -24331,10 +24322,13 @@
         <v>8</v>
       </c>
       <c r="H684" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="685" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I684">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="685" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A685" s="1">
         <v>46095</v>
       </c>
@@ -24359,8 +24353,11 @@
       <c r="H685" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="686" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I685">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="686" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A686" s="1">
         <v>46095</v>
       </c>
@@ -24374,7 +24371,7 @@
         <v>1064</v>
       </c>
       <c r="F686" t="s">
-        <v>1421</v>
+        <v>119</v>
       </c>
       <c r="G686" t="s">
         <v>8</v>
@@ -24382,8 +24379,11 @@
       <c r="H686" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="687" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I686">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="687" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A687" s="1">
         <v>46095</v>
       </c>
@@ -24406,10 +24406,13 @@
         <v>8</v>
       </c>
       <c r="H687" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="688" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I687">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="688" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A688" s="1">
         <v>46095</v>
       </c>
@@ -24434,8 +24437,11 @@
       <c r="H688" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="689" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I688">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="689" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A689" s="1">
         <v>46095</v>
       </c>
@@ -24458,10 +24464,13 @@
         <v>8</v>
       </c>
       <c r="H689" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="690" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I689">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="690" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A690" s="1">
         <v>46095</v>
       </c>
@@ -24486,8 +24495,11 @@
       <c r="H690" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="691" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I690">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="691" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A691" s="1">
         <v>46095</v>
       </c>
@@ -24510,10 +24522,13 @@
         <v>8</v>
       </c>
       <c r="H691" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="692" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I691">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="692" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A692" s="1">
         <v>46095</v>
       </c>
@@ -24538,8 +24553,11 @@
       <c r="H692" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="693" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I692">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A693" s="1">
         <v>46095</v>
       </c>
@@ -24562,10 +24580,13 @@
         <v>8</v>
       </c>
       <c r="H693" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="694" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I693">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="694" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A694" s="1">
         <v>46097</v>
       </c>
@@ -24575,6 +24596,12 @@
       <c r="C694" t="s">
         <v>1441</v>
       </c>
+      <c r="D694" t="s">
+        <v>1250</v>
+      </c>
+      <c r="E694" t="s">
+        <v>1062</v>
+      </c>
       <c r="F694" t="s">
         <v>16</v>
       </c>
@@ -24584,8 +24611,11 @@
       <c r="H694" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="695" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I694">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="695" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A695" s="1">
         <v>46097</v>
       </c>
@@ -24595,6 +24625,12 @@
       <c r="C695" t="s">
         <v>1443</v>
       </c>
+      <c r="D695" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E695" t="s">
+        <v>1062</v>
+      </c>
       <c r="F695" t="s">
         <v>17</v>
       </c>
@@ -24604,8 +24640,11 @@
       <c r="H695" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="696" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I695">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="696" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A696" s="1">
         <v>46097</v>
       </c>
@@ -24615,22 +24654,40 @@
       <c r="C696" t="s">
         <v>1445</v>
       </c>
+      <c r="D696" t="s">
+        <v>1250</v>
+      </c>
+      <c r="E696" t="s">
+        <v>1062</v>
+      </c>
       <c r="F696" t="s">
-        <v>1446</v>
+        <v>47</v>
+      </c>
+      <c r="G696" t="s">
+        <v>8</v>
       </c>
       <c r="H696" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="697" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I696">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="697" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A697" s="1">
         <v>46097</v>
       </c>
       <c r="B697" t="s">
+        <v>1446</v>
+      </c>
+      <c r="C697" t="s">
         <v>1447</v>
       </c>
-      <c r="C697" t="s">
-        <v>1448</v>
+      <c r="D697" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E697" t="s">
+        <v>1062</v>
       </c>
       <c r="F697" t="s">
         <v>17</v>
@@ -24641,16 +24698,25 @@
       <c r="H697" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="698" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I697">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A698" s="1">
         <v>46097</v>
       </c>
       <c r="B698" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C698" t="s">
         <v>1449</v>
       </c>
-      <c r="C698" t="s">
-        <v>1450</v>
+      <c r="D698" t="s">
+        <v>1250</v>
+      </c>
+      <c r="E698" t="s">
+        <v>1062</v>
       </c>
       <c r="F698" t="s">
         <v>16</v>
@@ -24660,6 +24726,9 @@
       </c>
       <c r="H698" t="s">
         <v>19</v>
+      </c>
+      <c r="I698">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated balde and producao - base 23/03/2026
</commit_message>
<xml_diff>
--- a/first-atlas/producao_2026-03.xlsx
+++ b/first-atlas/producao_2026-03.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\augustoalmeida\Augusto\bots_comissionamento\bot_atlas\first-atlas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B133BA-F564-4FFE-BB71-FDCE634A43DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BFD83C1-3397-4FAD-BB53-808214428643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F5572131-3C84-4D9C-B555-72DCC3B1940B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7157" uniqueCount="2081">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7663" uniqueCount="2272">
   <si>
     <t>DATA_BASE</t>
   </si>
@@ -6282,6 +6282,579 @@
   </si>
   <si>
     <t>Ata de eleicao da empresa ASSOCIACAO ESCOLINHA FUNDAMENTOS DO FUTEBOL, atualizado e registrada no orgao competente. Esse documento formaliza a eleicao e/ou nomeacao dos representantes legais e administradores, informando cargos, prazos de mandato e poderes de representacao, comprovando quem esta autorizado a agir em nome da entidade.&lt;br&gt;&lt;br&gt;Estatuto social da empresa ASSOCIACAO ESCOLINHA FUNDAMENTOS DO FUTEBOL, atualizado e registrado no orgao competente. Esse documento estabelece as regras de funcionamento da empresa, descrevendo sua finalidade, estrutura administrativa, orgaos de gestao e forma de representacao legal, comprovando sua existencia e regularidade.</t>
+  </si>
+  <si>
+    <t>31868637000128</t>
+  </si>
+  <si>
+    <t>42063902000117</t>
+  </si>
+  <si>
+    <t>52247270000103</t>
+  </si>
+  <si>
+    <t>62161364000100</t>
+  </si>
+  <si>
+    <t>59218814000140</t>
+  </si>
+  <si>
+    <t>07530434000142</t>
+  </si>
+  <si>
+    <t>58488593000167</t>
+  </si>
+  <si>
+    <t>62691113000138</t>
+  </si>
+  <si>
+    <t>48521770000106</t>
+  </si>
+  <si>
+    <t>21738366000132</t>
+  </si>
+  <si>
+    <t>17659973000130</t>
+  </si>
+  <si>
+    <t>22028750000104</t>
+  </si>
+  <si>
+    <t>47925982000196</t>
+  </si>
+  <si>
+    <t>55220635000196</t>
+  </si>
+  <si>
+    <t>36044844000181</t>
+  </si>
+  <si>
+    <t>61298260000180</t>
+  </si>
+  <si>
+    <t>54006045000100</t>
+  </si>
+  <si>
+    <t>59792053000135</t>
+  </si>
+  <si>
+    <t>58740619000201</t>
+  </si>
+  <si>
+    <t>47051883000122</t>
+  </si>
+  <si>
+    <t>52699450000118</t>
+  </si>
+  <si>
+    <t>59791910000182</t>
+  </si>
+  <si>
+    <t>43344176000173</t>
+  </si>
+  <si>
+    <t>17671515000116</t>
+  </si>
+  <si>
+    <t>00192878000176</t>
+  </si>
+  <si>
+    <t>09107200000112</t>
+  </si>
+  <si>
+    <t>26875809000150</t>
+  </si>
+  <si>
+    <t>64114216000160</t>
+  </si>
+  <si>
+    <t>17353487000199</t>
+  </si>
+  <si>
+    <t>60305011000101</t>
+  </si>
+  <si>
+    <t>38891070000150</t>
+  </si>
+  <si>
+    <t>47535579000150</t>
+  </si>
+  <si>
+    <t>28537790000249</t>
+  </si>
+  <si>
+    <t>42430521000129</t>
+  </si>
+  <si>
+    <t>11916506000161</t>
+  </si>
+  <si>
+    <t>36448699000102</t>
+  </si>
+  <si>
+    <t>53214837000108</t>
+  </si>
+  <si>
+    <t>45280899000181</t>
+  </si>
+  <si>
+    <t>64726336000119</t>
+  </si>
+  <si>
+    <t>46592778000138</t>
+  </si>
+  <si>
+    <t>64666153000155</t>
+  </si>
+  <si>
+    <t>15231029000151</t>
+  </si>
+  <si>
+    <t>26078145000107</t>
+  </si>
+  <si>
+    <t>64916272000119</t>
+  </si>
+  <si>
+    <t>60441695000179</t>
+  </si>
+  <si>
+    <t>52270574000183</t>
+  </si>
+  <si>
+    <t>09622925000149</t>
+  </si>
+  <si>
+    <t>65105661000127</t>
+  </si>
+  <si>
+    <t>38981445000172</t>
+  </si>
+  <si>
+    <t>60282404000147</t>
+  </si>
+  <si>
+    <t>59937472000118</t>
+  </si>
+  <si>
+    <t>61527450000121</t>
+  </si>
+  <si>
+    <t>32915024000167</t>
+  </si>
+  <si>
+    <t>47281884000163</t>
+  </si>
+  <si>
+    <t>60835621000117</t>
+  </si>
+  <si>
+    <t>64369662000116</t>
+  </si>
+  <si>
+    <t>44457840000153</t>
+  </si>
+  <si>
+    <t>32315559000288</t>
+  </si>
+  <si>
+    <t>61414103000192</t>
+  </si>
+  <si>
+    <t>51916183000120</t>
+  </si>
+  <si>
+    <t>09425553000160</t>
+  </si>
+  <si>
+    <t>49828832000190</t>
+  </si>
+  <si>
+    <t>PONTO DO TERERE LTDA</t>
+  </si>
+  <si>
+    <t>Raphael Ferreira Jacintho</t>
+  </si>
+  <si>
+    <t>60533126000153</t>
+  </si>
+  <si>
+    <t>PAINEIS EM LED H S PUBLICIDADE E PROPAGANDA LTDA</t>
+  </si>
+  <si>
+    <t>53139827000147</t>
+  </si>
+  <si>
+    <t>MC TECH ENGENHARIA LTDA</t>
+  </si>
+  <si>
+    <t>65716951000107</t>
+  </si>
+  <si>
+    <t>BERTEC MANUTENCAO DE MAQUINAS INDUSTRIAIS LTDA</t>
+  </si>
+  <si>
+    <t>64269100000109</t>
+  </si>
+  <si>
+    <t>GHF LOCACOES E TRANSPORTES LTDA</t>
+  </si>
+  <si>
+    <t>63183977000101</t>
+  </si>
+  <si>
+    <t>KJ DRINKS VIDA LTDA</t>
+  </si>
+  <si>
+    <t>30698034000162</t>
+  </si>
+  <si>
+    <t>REIS AUTO CENTER LTDA</t>
+  </si>
+  <si>
+    <t>59617054000143</t>
+  </si>
+  <si>
+    <t>PADUA ASSUNCAO LTDA</t>
+  </si>
+  <si>
+    <t>63439209000176</t>
+  </si>
+  <si>
+    <t>ACF TRANSPORTADORA URUPES LTDA</t>
+  </si>
+  <si>
+    <t>61317826000173</t>
+  </si>
+  <si>
+    <t>PE DE PANO MATERIAL DE CONSTRUCAO LTDA</t>
+  </si>
+  <si>
+    <t>17901115000150</t>
+  </si>
+  <si>
+    <t>TROPICAL MIX PRODUTOS PARA SORVETES EXPRESSO LTDA</t>
+  </si>
+  <si>
+    <t>10419748000187</t>
+  </si>
+  <si>
+    <t>RENFE INDUSTRIA E COMERCIO DE CONFECCOES LTDA</t>
+  </si>
+  <si>
+    <t>23973310000198</t>
+  </si>
+  <si>
+    <t>23.973.310 ROBSON BARBOZA VITERALE</t>
+  </si>
+  <si>
+    <t>12861245000192</t>
+  </si>
+  <si>
+    <t>ETERNOS TRAJES LTDA</t>
+  </si>
+  <si>
+    <t>62963203000130</t>
+  </si>
+  <si>
+    <t>MF AUTOMACAO LTDA</t>
+  </si>
+  <si>
+    <t>27970421000100</t>
+  </si>
+  <si>
+    <t>SUCATAS MAIA LTDA</t>
+  </si>
+  <si>
+    <t>52922100000179</t>
+  </si>
+  <si>
+    <t>RECONS OBRAS LTDA</t>
+  </si>
+  <si>
+    <t>61153190000171</t>
+  </si>
+  <si>
+    <t>LEON PRE FABRICADOS DE CONCRETO LTDA</t>
+  </si>
+  <si>
+    <t>60252607000190</t>
+  </si>
+  <si>
+    <t>UNIPLAY COMERCIO E IMPORTACAO DE BRINQUEDOS LTDA</t>
+  </si>
+  <si>
+    <t>19509903000120</t>
+  </si>
+  <si>
+    <t>M.Z AUTO PECAS LATAS E ACESSORIOS LTDA</t>
+  </si>
+  <si>
+    <t>17850958000174</t>
+  </si>
+  <si>
+    <t>CIDAUTOMOVEIS OFICINA MECANICA LTDA</t>
+  </si>
+  <si>
+    <t>61804342000159</t>
+  </si>
+  <si>
+    <t>RESOUDRE CONSULTORIA LTDA</t>
+  </si>
+  <si>
+    <t>64922299000114</t>
+  </si>
+  <si>
+    <t>DS MOREIRA COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>51763005000107</t>
+  </si>
+  <si>
+    <t>51.763.005 OSVALDO APARECIDO RODRIGUES TEIXEIRA</t>
+  </si>
+  <si>
+    <t>12230174000120</t>
+  </si>
+  <si>
+    <t>ESPACO LA BELLA LTDA</t>
+  </si>
+  <si>
+    <t>17457965000100</t>
+  </si>
+  <si>
+    <t>RESTAURANTE CANOAS LTDA</t>
+  </si>
+  <si>
+    <t>22321196000159</t>
+  </si>
+  <si>
+    <t>VIDRACARIA VD LTDA</t>
+  </si>
+  <si>
+    <t>48498515000190</t>
+  </si>
+  <si>
+    <t>RUBEM ISMAEL VASQUES</t>
+  </si>
+  <si>
+    <t>33095016000184</t>
+  </si>
+  <si>
+    <t>VIANEY RODRIGUES DE ALEXANDRIA</t>
+  </si>
+  <si>
+    <t>60673056000139</t>
+  </si>
+  <si>
+    <t>LUEDE CONFECCOES LTDA</t>
+  </si>
+  <si>
+    <t>32499745000133</t>
+  </si>
+  <si>
+    <t>GISLAINE DA SILVA LIMA</t>
+  </si>
+  <si>
+    <t>37576393000196</t>
+  </si>
+  <si>
+    <t>CARLA DE CARVALHO CAMPOS SOARES</t>
+  </si>
+  <si>
+    <t>62343534000178</t>
+  </si>
+  <si>
+    <t>62.343.534 DJEISON ASSUNCAO DA SILVA</t>
+  </si>
+  <si>
+    <t>49184636000120</t>
+  </si>
+  <si>
+    <t>49.184.636 JULIO DE SOUZA PINTO</t>
+  </si>
+  <si>
+    <t>65010763000169</t>
+  </si>
+  <si>
+    <t>ANDERSON OLIVEIRA DOS SANTOS SOCIEDADE INDIVIDUAL DE ADVOCACIA</t>
+  </si>
+  <si>
+    <t>49298069000132</t>
+  </si>
+  <si>
+    <t>49.298.069 JOAO CARLOS RIBEIRO MUNIZ</t>
+  </si>
+  <si>
+    <t>23161597000151</t>
+  </si>
+  <si>
+    <t>MARIA ERICA PEREIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>59982299000170</t>
+  </si>
+  <si>
+    <t>LEVY PNEUS E RODAS LTDA</t>
+  </si>
+  <si>
+    <t>59126525000110</t>
+  </si>
+  <si>
+    <t>JK ATACAREJO DE MODAS E ACESSORIOS LTDA</t>
+  </si>
+  <si>
+    <t>40876870000305</t>
+  </si>
+  <si>
+    <t>S. C. DIAS DE OLIVEIRA LTDA</t>
+  </si>
+  <si>
+    <t>21944626000126</t>
+  </si>
+  <si>
+    <t>ZOOM PLAMOVEIS AMBIENTES PLANEJADOS LTDA</t>
+  </si>
+  <si>
+    <t>45551481000161</t>
+  </si>
+  <si>
+    <t>NICHOLLAS LAWER CANHET VIDIGAL</t>
+  </si>
+  <si>
+    <t>52594547000166</t>
+  </si>
+  <si>
+    <t>JI SERVICOS DE INSTALACOES LTDA</t>
+  </si>
+  <si>
+    <t>43297729000184</t>
+  </si>
+  <si>
+    <t>PONTO DA SUCATA LTDA</t>
+  </si>
+  <si>
+    <t>36017615000178</t>
+  </si>
+  <si>
+    <t>MARIA TEREZINHA DIAS DA CUNHA</t>
+  </si>
+  <si>
+    <t>41346335000143</t>
+  </si>
+  <si>
+    <t>DISTRIBUIDORA DE CARNES SAO JUDAS TADEU LTDA</t>
+  </si>
+  <si>
+    <t>39712347000100</t>
+  </si>
+  <si>
+    <t>FERNANDO HENRIQUE FRANCA LTDA</t>
+  </si>
+  <si>
+    <t>Joao Pedro Mayer Ribeiro Oliveira</t>
+  </si>
+  <si>
+    <t>41406909000121</t>
+  </si>
+  <si>
+    <t>WELLINGTON RENATO BECA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>64336898000156</t>
+  </si>
+  <si>
+    <t>RESTAURANTE BOTECO GRILL LTDA</t>
+  </si>
+  <si>
+    <t>57842953000114</t>
+  </si>
+  <si>
+    <t>MANIA DE BICHO PET SHOP E CLINICA VETERINARIA LTDA</t>
+  </si>
+  <si>
+    <t>53206008000175</t>
+  </si>
+  <si>
+    <t>MARLIERE DE MELO JUNIOR LTDA</t>
+  </si>
+  <si>
+    <t>64106243000191</t>
+  </si>
+  <si>
+    <t>GOLL GRILL LANCHONETE LTDA</t>
+  </si>
+  <si>
+    <t>60110630000140</t>
+  </si>
+  <si>
+    <t>MARCELO F. RAMPAZZO LTDA</t>
+  </si>
+  <si>
+    <t>56960815000177</t>
+  </si>
+  <si>
+    <t>BARATINHA PIPAS COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>41697156000150</t>
+  </si>
+  <si>
+    <t>KWI CONSTRUCOES E REFORMAS LTDA</t>
+  </si>
+  <si>
+    <t>37636846000122</t>
+  </si>
+  <si>
+    <t>CRS EMPREITEIRA LTDA</t>
+  </si>
+  <si>
+    <t>50061409000196</t>
+  </si>
+  <si>
+    <t>50.061.409 DANIEL PEREIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>27620284000175</t>
+  </si>
+  <si>
+    <t>27.620.284 JEAN TIAGO PEREIRA</t>
+  </si>
+  <si>
+    <t>43803389000116</t>
+  </si>
+  <si>
+    <t>LINO'S CONFECCOES LTDA</t>
+  </si>
+  <si>
+    <t>Mensageria</t>
+  </si>
+  <si>
+    <t>42630233000118</t>
+  </si>
+  <si>
+    <t>ELSON AMARANTE CARDOSO</t>
+  </si>
+  <si>
+    <t>57380929000100</t>
+  </si>
+  <si>
+    <t>M FERNANDES TRANSPORTES LTDA</t>
+  </si>
+  <si>
+    <t>64054764000142</t>
+  </si>
+  <si>
+    <t>Empresa: VANGINER RODRIGUES DOS ANJOS SILVA</t>
+  </si>
+  <si>
+    <t>34718763000194</t>
+  </si>
+  <si>
+    <t>34.718.763 CARLOS ALBERTO FLORINDO OLIVEIRA</t>
+  </si>
+  <si>
+    <t>Ata de eleicao da empresa INSTITUTO VIDA MELHOR, atualizado e registrada no orgao competente. Esse documento formaliza a eleicao e/ou nomeacao dos representantes legais e administradores, informando cargos, prazos de mandato e poderes de representacao, comprovando quem esta autorizado a agir em nome da entidade.&lt;br&gt;&lt;br&gt;Estatuto social da empresa INSTITUTO VIDA MELHOR, atualizado e registrado no orgao competente. Esse documento estabelece as regras de funcionamento da empresa, descrevendo sua finalidade, estrutura administrativa, orgaos de gestao e forma de representacao legal, comprovando sua existencia e regularidade.</t>
   </si>
 </sst>
 </file>
@@ -6654,7 +7227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A45A88-3D17-4433-986A-11075963C36F}">
-  <dimension ref="A1:I1041"/>
+  <dimension ref="A1:I1104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -6919,7 +7492,7 @@
         <v>7</v>
       </c>
       <c r="H9" t="s">
-        <v>23</v>
+        <v>696</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -8875,7 +9448,7 @@
         <v>7</v>
       </c>
       <c r="H78" t="s">
-        <v>23</v>
+        <v>696</v>
       </c>
       <c r="I78">
         <v>0</v>
@@ -9191,7 +9764,7 @@
         <v>7</v>
       </c>
       <c r="H89" t="s">
-        <v>23</v>
+        <v>696</v>
       </c>
       <c r="I89">
         <v>0</v>
@@ -12263,7 +12836,7 @@
         <v>7</v>
       </c>
       <c r="H197" t="s">
-        <v>23</v>
+        <v>696</v>
       </c>
       <c r="I197">
         <v>0</v>
@@ -15402,7 +15975,7 @@
         <v>8</v>
       </c>
       <c r="H307" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I307">
         <v>0</v>
@@ -15779,7 +16352,7 @@
         <v>8</v>
       </c>
       <c r="H320" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I320">
         <v>0</v>
@@ -17965,7 +18538,7 @@
         <v>8</v>
       </c>
       <c r="H396" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I396">
         <v>0</v>
@@ -21452,7 +22025,7 @@
         <v>7</v>
       </c>
       <c r="H518" t="s">
-        <v>696</v>
+        <v>19</v>
       </c>
       <c r="I518">
         <v>0</v>
@@ -22844,7 +23417,7 @@
         <v>929</v>
       </c>
       <c r="H566" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I566">
         <v>0</v>
@@ -26281,7 +26854,7 @@
         <v>8</v>
       </c>
       <c r="H687" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="I687">
         <v>0</v>
@@ -28954,7 +29527,7 @@
         <v>8</v>
       </c>
       <c r="H780" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I780">
         <v>0</v>
@@ -31865,7 +32438,7 @@
         <v>8</v>
       </c>
       <c r="H881" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I881">
         <v>0</v>
@@ -33039,7 +33612,7 @@
         <v>8</v>
       </c>
       <c r="H922" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I922">
         <v>0</v>
@@ -33155,7 +33728,7 @@
         <v>8</v>
       </c>
       <c r="H926" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I926">
         <v>0</v>
@@ -33587,7 +34160,7 @@
         <v>8</v>
       </c>
       <c r="H941" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I941">
         <v>0</v>
@@ -33674,7 +34247,7 @@
         <v>8</v>
       </c>
       <c r="H944" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I944">
         <v>0</v>
@@ -33761,7 +34334,10 @@
         <v>7</v>
       </c>
       <c r="H947" t="s">
-        <v>21</v>
+        <v>23</v>
+      </c>
+      <c r="I947">
+        <v>0</v>
       </c>
     </row>
     <row r="948" spans="1:9" x14ac:dyDescent="0.25">
@@ -33983,6 +34559,9 @@
       <c r="H955" t="s">
         <v>19</v>
       </c>
+      <c r="I955">
+        <v>0</v>
+      </c>
     </row>
     <row r="956" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A956" s="1">
@@ -34006,6 +34585,9 @@
       <c r="H956" t="s">
         <v>19</v>
       </c>
+      <c r="I956">
+        <v>0</v>
+      </c>
     </row>
     <row r="957" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A957" s="1">
@@ -34029,6 +34611,9 @@
       <c r="H957" t="s">
         <v>19</v>
       </c>
+      <c r="I957">
+        <v>0</v>
+      </c>
     </row>
     <row r="958" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A958" s="1">
@@ -34052,6 +34637,9 @@
       <c r="H958" t="s">
         <v>19</v>
       </c>
+      <c r="I958">
+        <v>0</v>
+      </c>
     </row>
     <row r="959" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A959" s="1">
@@ -34075,6 +34663,9 @@
       <c r="H959" t="s">
         <v>19</v>
       </c>
+      <c r="I959">
+        <v>0</v>
+      </c>
     </row>
     <row r="960" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A960" s="1">
@@ -34098,13 +34689,16 @@
       <c r="H960" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="961" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I960">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="961" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A961" s="1">
         <v>46101</v>
       </c>
-      <c r="B961">
-        <v>31868637000128</v>
+      <c r="B961" t="s">
+        <v>2081</v>
       </c>
       <c r="C961" t="s">
         <v>1984</v>
@@ -34122,15 +34716,18 @@
         <v>7</v>
       </c>
       <c r="H961" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="962" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I961">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="962" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A962" s="1">
         <v>46101</v>
       </c>
-      <c r="B962">
-        <v>42063902000117</v>
+      <c r="B962" t="s">
+        <v>2082</v>
       </c>
       <c r="C962" t="s">
         <v>1985</v>
@@ -34148,15 +34745,18 @@
         <v>8</v>
       </c>
       <c r="H962" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="963" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I962">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="963" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A963" s="1">
         <v>46101</v>
       </c>
-      <c r="B963">
-        <v>52247270000103</v>
+      <c r="B963" t="s">
+        <v>2083</v>
       </c>
       <c r="C963" t="s">
         <v>1986</v>
@@ -34176,13 +34776,16 @@
       <c r="H963" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="964" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I963">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="964" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A964" s="1">
         <v>46101</v>
       </c>
-      <c r="B964">
-        <v>62161364000100</v>
+      <c r="B964" t="s">
+        <v>2084</v>
       </c>
       <c r="C964" t="s">
         <v>1987</v>
@@ -34202,13 +34805,16 @@
       <c r="H964" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="965" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I964">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="965" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A965" s="1">
         <v>46101</v>
       </c>
-      <c r="B965">
-        <v>59218814000140</v>
+      <c r="B965" t="s">
+        <v>2085</v>
       </c>
       <c r="C965" t="s">
         <v>1988</v>
@@ -34228,13 +34834,16 @@
       <c r="H965" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="966" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I965">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="966" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A966" s="1">
         <v>46101</v>
       </c>
-      <c r="B966">
-        <v>7530434000142</v>
+      <c r="B966" t="s">
+        <v>2086</v>
       </c>
       <c r="C966" t="s">
         <v>1989</v>
@@ -34252,15 +34861,18 @@
         <v>7</v>
       </c>
       <c r="H966" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="967" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I966">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="967" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A967" s="1">
         <v>46101</v>
       </c>
-      <c r="B967">
-        <v>58488593000167</v>
+      <c r="B967" t="s">
+        <v>2087</v>
       </c>
       <c r="C967" t="s">
         <v>1990</v>
@@ -34280,13 +34892,16 @@
       <c r="H967" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="968" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I967">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="968" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A968" s="1">
         <v>46101</v>
       </c>
-      <c r="B968">
-        <v>62691113000138</v>
+      <c r="B968" t="s">
+        <v>2088</v>
       </c>
       <c r="C968" t="s">
         <v>1991</v>
@@ -34304,15 +34919,18 @@
         <v>8</v>
       </c>
       <c r="H968" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="969" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I968">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="969" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A969" s="1">
         <v>46101</v>
       </c>
-      <c r="B969">
-        <v>48521770000106</v>
+      <c r="B969" t="s">
+        <v>2089</v>
       </c>
       <c r="C969" t="s">
         <v>1992</v>
@@ -34332,13 +34950,16 @@
       <c r="H969" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="970" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I969">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="970" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A970" s="1">
         <v>46101</v>
       </c>
-      <c r="B970">
-        <v>21738366000132</v>
+      <c r="B970" t="s">
+        <v>2090</v>
       </c>
       <c r="C970" t="s">
         <v>1993</v>
@@ -34358,13 +34979,16 @@
       <c r="H970" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="971" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I970">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="971" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A971" s="1">
         <v>46101</v>
       </c>
-      <c r="B971">
-        <v>17659973000130</v>
+      <c r="B971" t="s">
+        <v>2091</v>
       </c>
       <c r="C971" t="s">
         <v>1994</v>
@@ -34384,13 +35008,16 @@
       <c r="H971" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="972" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I971">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="972" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A972" s="1">
         <v>46101</v>
       </c>
-      <c r="B972">
-        <v>22028750000104</v>
+      <c r="B972" t="s">
+        <v>2092</v>
       </c>
       <c r="C972" t="s">
         <v>1995</v>
@@ -34410,13 +35037,16 @@
       <c r="H972" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="973" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I972">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="973" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A973" s="1">
         <v>46101</v>
       </c>
-      <c r="B973">
-        <v>47925982000196</v>
+      <c r="B973" t="s">
+        <v>2093</v>
       </c>
       <c r="C973" t="s">
         <v>1996</v>
@@ -34436,13 +35066,16 @@
       <c r="H973" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="974" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I973">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="974" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A974" s="1">
         <v>46101</v>
       </c>
-      <c r="B974">
-        <v>55220635000196</v>
+      <c r="B974" t="s">
+        <v>2094</v>
       </c>
       <c r="C974" t="s">
         <v>1036</v>
@@ -34462,13 +35095,16 @@
       <c r="H974" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="975" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I974" t="s">
+        <v>2271</v>
+      </c>
+    </row>
+    <row r="975" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A975" s="1">
         <v>46101</v>
       </c>
-      <c r="B975">
-        <v>36044844000181</v>
+      <c r="B975" t="s">
+        <v>2095</v>
       </c>
       <c r="C975" t="s">
         <v>1997</v>
@@ -34488,13 +35124,16 @@
       <c r="H975" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="976" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I975">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="976" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A976" s="1">
         <v>46101</v>
       </c>
-      <c r="B976">
-        <v>61298260000180</v>
+      <c r="B976" t="s">
+        <v>2096</v>
       </c>
       <c r="C976" t="s">
         <v>1998</v>
@@ -34514,13 +35153,16 @@
       <c r="H976" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="977" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I976">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="977" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A977" s="1">
         <v>46101</v>
       </c>
-      <c r="B977">
-        <v>54006045000100</v>
+      <c r="B977" t="s">
+        <v>2097</v>
       </c>
       <c r="C977" t="s">
         <v>1999</v>
@@ -34540,13 +35182,16 @@
       <c r="H977" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="978" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I977">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="978" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A978" s="1">
         <v>46101</v>
       </c>
-      <c r="B978">
-        <v>59792053000135</v>
+      <c r="B978" t="s">
+        <v>2098</v>
       </c>
       <c r="C978" t="s">
         <v>2000</v>
@@ -34566,13 +35211,16 @@
       <c r="H978" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="979" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I978">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="979" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A979" s="1">
         <v>46101</v>
       </c>
-      <c r="B979">
-        <v>58740619000201</v>
+      <c r="B979" t="s">
+        <v>2099</v>
       </c>
       <c r="C979" t="s">
         <v>2001</v>
@@ -34590,15 +35238,18 @@
         <v>8</v>
       </c>
       <c r="H979" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="980" spans="1:8" x14ac:dyDescent="0.25">
+        <v>696</v>
+      </c>
+      <c r="I979">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="980" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A980" s="1">
         <v>46101</v>
       </c>
-      <c r="B980">
-        <v>47051883000122</v>
+      <c r="B980" t="s">
+        <v>2100</v>
       </c>
       <c r="C980" t="s">
         <v>803</v>
@@ -34616,15 +35267,18 @@
         <v>13</v>
       </c>
       <c r="H980" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="981" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I980">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="981" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A981" s="1">
         <v>46101</v>
       </c>
-      <c r="B981">
-        <v>52699450000118</v>
+      <c r="B981" t="s">
+        <v>2101</v>
       </c>
       <c r="C981" t="s">
         <v>2002</v>
@@ -34642,15 +35296,18 @@
         <v>8</v>
       </c>
       <c r="H981" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="982" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I981">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="982" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A982" s="1">
         <v>46101</v>
       </c>
-      <c r="B982">
-        <v>59791910000182</v>
+      <c r="B982" t="s">
+        <v>2102</v>
       </c>
       <c r="C982" t="s">
         <v>2003</v>
@@ -34668,15 +35325,18 @@
         <v>7</v>
       </c>
       <c r="H982" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="983" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I982">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="983" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A983" s="1">
         <v>46101</v>
       </c>
-      <c r="B983">
-        <v>43344176000173</v>
+      <c r="B983" t="s">
+        <v>2103</v>
       </c>
       <c r="C983" t="s">
         <v>2004</v>
@@ -34696,13 +35356,16 @@
       <c r="H983" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="984" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I983">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="984" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A984" s="1">
         <v>46101</v>
       </c>
-      <c r="B984">
-        <v>17671515000116</v>
+      <c r="B984" t="s">
+        <v>2104</v>
       </c>
       <c r="C984" t="s">
         <v>2005</v>
@@ -34723,12 +35386,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="985" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="985" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A985" s="1">
         <v>46101</v>
       </c>
-      <c r="B985">
-        <v>192878000176</v>
+      <c r="B985" t="s">
+        <v>2105</v>
       </c>
       <c r="C985" t="s">
         <v>2006</v>
@@ -34746,15 +35409,18 @@
         <v>7</v>
       </c>
       <c r="H985" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="986" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I985">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="986" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A986" s="1">
         <v>46101</v>
       </c>
-      <c r="B986">
-        <v>9107200000112</v>
+      <c r="B986" t="s">
+        <v>2106</v>
       </c>
       <c r="C986" t="s">
         <v>2007</v>
@@ -34774,13 +35440,16 @@
       <c r="H986" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="987" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I986">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="987" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A987" s="1">
         <v>46101</v>
       </c>
-      <c r="B987">
-        <v>26875809000150</v>
+      <c r="B987" t="s">
+        <v>2107</v>
       </c>
       <c r="C987" t="s">
         <v>2008</v>
@@ -34800,13 +35469,16 @@
       <c r="H987" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="988" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I987">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="988" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A988" s="1">
         <v>46101</v>
       </c>
-      <c r="B988">
-        <v>64114216000160</v>
+      <c r="B988" t="s">
+        <v>2108</v>
       </c>
       <c r="C988" t="s">
         <v>2009</v>
@@ -34826,13 +35498,16 @@
       <c r="H988" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="989" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I988">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="989" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A989" s="1">
         <v>46101</v>
       </c>
-      <c r="B989">
-        <v>17353487000199</v>
+      <c r="B989" t="s">
+        <v>2109</v>
       </c>
       <c r="C989" t="s">
         <v>2011</v>
@@ -34850,15 +35525,18 @@
         <v>7</v>
       </c>
       <c r="H989" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="990" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I989">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="990" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A990" s="1">
         <v>46101</v>
       </c>
-      <c r="B990">
-        <v>60305011000101</v>
+      <c r="B990" t="s">
+        <v>2110</v>
       </c>
       <c r="C990" t="s">
         <v>2012</v>
@@ -34876,15 +35554,18 @@
         <v>8</v>
       </c>
       <c r="H990" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="991" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I990">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="991" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A991" s="1">
         <v>46101</v>
       </c>
-      <c r="B991">
-        <v>38891070000150</v>
+      <c r="B991" t="s">
+        <v>2111</v>
       </c>
       <c r="C991" t="s">
         <v>2013</v>
@@ -34902,15 +35583,18 @@
         <v>8</v>
       </c>
       <c r="H991" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="992" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I991" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="992" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A992" s="1">
         <v>46101</v>
       </c>
-      <c r="B992">
-        <v>47535579000150</v>
+      <c r="B992" t="s">
+        <v>2112</v>
       </c>
       <c r="C992" t="s">
         <v>2014</v>
@@ -34930,13 +35614,16 @@
       <c r="H992" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="993" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I992">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="993" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A993" s="1">
         <v>46101</v>
       </c>
-      <c r="B993">
-        <v>28537790000249</v>
+      <c r="B993" t="s">
+        <v>2113</v>
       </c>
       <c r="C993" t="s">
         <v>2015</v>
@@ -34954,15 +35641,18 @@
         <v>7</v>
       </c>
       <c r="H993" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="994" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I993">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="994" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A994" s="1">
         <v>46101</v>
       </c>
-      <c r="B994">
-        <v>42430521000129</v>
+      <c r="B994" t="s">
+        <v>2114</v>
       </c>
       <c r="C994" t="s">
         <v>2016</v>
@@ -34980,15 +35670,18 @@
         <v>7</v>
       </c>
       <c r="H994" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="995" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I994">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="995" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A995" s="1">
         <v>46101</v>
       </c>
-      <c r="B995">
-        <v>11916506000161</v>
+      <c r="B995" t="s">
+        <v>2115</v>
       </c>
       <c r="C995" t="s">
         <v>922</v>
@@ -35008,13 +35701,16 @@
       <c r="H995" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="996" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I995">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="996" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A996" s="1">
         <v>46101</v>
       </c>
-      <c r="B996">
-        <v>36448699000102</v>
+      <c r="B996" t="s">
+        <v>2116</v>
       </c>
       <c r="C996" t="s">
         <v>2017</v>
@@ -35034,13 +35730,16 @@
       <c r="H996" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="997" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I996">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="997" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A997" s="1">
         <v>46101</v>
       </c>
-      <c r="B997">
-        <v>53214837000108</v>
+      <c r="B997" t="s">
+        <v>2117</v>
       </c>
       <c r="C997" t="s">
         <v>2018</v>
@@ -35060,13 +35759,16 @@
       <c r="H997" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="998" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I997">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="998" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A998" s="1">
         <v>46101</v>
       </c>
-      <c r="B998">
-        <v>45280899000181</v>
+      <c r="B998" t="s">
+        <v>2118</v>
       </c>
       <c r="C998" t="s">
         <v>2019</v>
@@ -35084,15 +35786,18 @@
         <v>7</v>
       </c>
       <c r="H998" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="999" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I998">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="999" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A999" s="1">
         <v>46101</v>
       </c>
-      <c r="B999">
-        <v>64726336000119</v>
+      <c r="B999" t="s">
+        <v>2119</v>
       </c>
       <c r="C999" t="s">
         <v>2020</v>
@@ -35112,13 +35817,16 @@
       <c r="H999" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="1000" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I999">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1000" s="1">
         <v>46101</v>
       </c>
-      <c r="B1000">
-        <v>46592778000138</v>
+      <c r="B1000" t="s">
+        <v>2120</v>
       </c>
       <c r="C1000" t="s">
         <v>2021</v>
@@ -35136,15 +35844,18 @@
         <v>8</v>
       </c>
       <c r="H1000" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1001" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1000">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1001" s="1">
         <v>46101</v>
       </c>
-      <c r="B1001">
-        <v>64666153000155</v>
+      <c r="B1001" t="s">
+        <v>2121</v>
       </c>
       <c r="C1001" t="s">
         <v>2022</v>
@@ -35162,15 +35873,18 @@
         <v>8</v>
       </c>
       <c r="H1001" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1002" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1001">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1002" s="1">
         <v>46101</v>
       </c>
-      <c r="B1002">
-        <v>15231029000151</v>
+      <c r="B1002" t="s">
+        <v>2122</v>
       </c>
       <c r="C1002" t="s">
         <v>2023</v>
@@ -35190,13 +35904,16 @@
       <c r="H1002" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1003" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1002">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1003" s="1">
         <v>46101</v>
       </c>
-      <c r="B1003">
-        <v>26078145000107</v>
+      <c r="B1003" t="s">
+        <v>2123</v>
       </c>
       <c r="C1003" t="s">
         <v>2024</v>
@@ -35216,13 +35933,16 @@
       <c r="H1003" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1004" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1003">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1004" s="1">
         <v>46101</v>
       </c>
-      <c r="B1004">
-        <v>64916272000119</v>
+      <c r="B1004" t="s">
+        <v>2124</v>
       </c>
       <c r="C1004" t="s">
         <v>2025</v>
@@ -35240,15 +35960,18 @@
         <v>7</v>
       </c>
       <c r="H1004" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="1005" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1004">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1005" s="1">
         <v>46101</v>
       </c>
-      <c r="B1005">
-        <v>60441695000179</v>
+      <c r="B1005" t="s">
+        <v>2125</v>
       </c>
       <c r="C1005" t="s">
         <v>2026</v>
@@ -35266,15 +35989,18 @@
         <v>7</v>
       </c>
       <c r="H1005" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1006" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I1005">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1006" s="1">
         <v>46101</v>
       </c>
-      <c r="B1006">
-        <v>52270574000183</v>
+      <c r="B1006" t="s">
+        <v>2126</v>
       </c>
       <c r="C1006" t="s">
         <v>2027</v>
@@ -35292,15 +36018,18 @@
         <v>8</v>
       </c>
       <c r="H1006" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1007" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I1006">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1007" s="1">
         <v>46101</v>
       </c>
-      <c r="B1007">
-        <v>9622925000149</v>
+      <c r="B1007" t="s">
+        <v>2127</v>
       </c>
       <c r="C1007" t="s">
         <v>2028</v>
@@ -35320,13 +36049,16 @@
       <c r="H1007" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1008" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1007">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1008" s="1">
         <v>46101</v>
       </c>
-      <c r="B1008">
-        <v>65105661000127</v>
+      <c r="B1008" t="s">
+        <v>2128</v>
       </c>
       <c r="C1008" t="s">
         <v>2029</v>
@@ -35344,15 +36076,18 @@
         <v>7</v>
       </c>
       <c r="H1008" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1009" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I1008">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1009" s="1">
         <v>46101</v>
       </c>
-      <c r="B1009">
-        <v>38981445000172</v>
+      <c r="B1009" t="s">
+        <v>2129</v>
       </c>
       <c r="C1009" t="s">
         <v>2030</v>
@@ -35372,13 +36107,16 @@
       <c r="H1009" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1010" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1009">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1010" s="1">
         <v>46101</v>
       </c>
-      <c r="B1010">
-        <v>60282404000147</v>
+      <c r="B1010" t="s">
+        <v>2130</v>
       </c>
       <c r="C1010" t="s">
         <v>2031</v>
@@ -35396,15 +36134,18 @@
         <v>10</v>
       </c>
       <c r="H1010" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1011" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I1010">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1011" s="1">
         <v>46101</v>
       </c>
-      <c r="B1011">
-        <v>59937472000118</v>
+      <c r="B1011" t="s">
+        <v>2131</v>
       </c>
       <c r="C1011" t="s">
         <v>2032</v>
@@ -35424,13 +36165,16 @@
       <c r="H1011" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1012" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1011">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1012" s="1">
         <v>46101</v>
       </c>
-      <c r="B1012">
-        <v>61527450000121</v>
+      <c r="B1012" t="s">
+        <v>2132</v>
       </c>
       <c r="C1012" t="s">
         <v>2033</v>
@@ -35450,13 +36194,16 @@
       <c r="H1012" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1013" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1012">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1013" s="1">
         <v>46101</v>
       </c>
-      <c r="B1013">
-        <v>32915024000167</v>
+      <c r="B1013" t="s">
+        <v>2133</v>
       </c>
       <c r="C1013" t="s">
         <v>2034</v>
@@ -35474,15 +36221,15 @@
         <v>7</v>
       </c>
       <c r="H1013" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="1014" spans="1:8" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1014" s="1">
         <v>46101</v>
       </c>
-      <c r="B1014">
-        <v>47281884000163</v>
+      <c r="B1014" t="s">
+        <v>2134</v>
       </c>
       <c r="C1014" t="s">
         <v>2035</v>
@@ -35502,13 +36249,16 @@
       <c r="H1014" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="1015" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1014">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1015" s="1">
         <v>46101</v>
       </c>
-      <c r="B1015">
-        <v>60835621000117</v>
+      <c r="B1015" t="s">
+        <v>2135</v>
       </c>
       <c r="C1015" t="s">
         <v>2036</v>
@@ -35528,13 +36278,16 @@
       <c r="H1015" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="1016" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1015">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1016" s="1">
         <v>46101</v>
       </c>
-      <c r="B1016">
-        <v>64369662000116</v>
+      <c r="B1016" t="s">
+        <v>2136</v>
       </c>
       <c r="C1016" t="s">
         <v>1114</v>
@@ -35552,15 +36305,18 @@
         <v>7</v>
       </c>
       <c r="H1016" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1017" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1016">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1017" s="1">
         <v>46101</v>
       </c>
-      <c r="B1017">
-        <v>44457840000153</v>
+      <c r="B1017" t="s">
+        <v>2137</v>
       </c>
       <c r="C1017" t="s">
         <v>2037</v>
@@ -35578,15 +36334,18 @@
         <v>13</v>
       </c>
       <c r="H1017" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1018" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I1017" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1018" s="1">
         <v>46101</v>
       </c>
-      <c r="B1018">
-        <v>32315559000288</v>
+      <c r="B1018" t="s">
+        <v>2138</v>
       </c>
       <c r="C1018" t="s">
         <v>2038</v>
@@ -35604,15 +36363,15 @@
         <v>8</v>
       </c>
       <c r="H1018" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1019" spans="1:8" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1019" s="1">
         <v>46101</v>
       </c>
-      <c r="B1019">
-        <v>61414103000192</v>
+      <c r="B1019" t="s">
+        <v>2139</v>
       </c>
       <c r="C1019" t="s">
         <v>2039</v>
@@ -35632,13 +36391,16 @@
       <c r="H1019" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1020" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1019">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1020" s="1">
         <v>46101</v>
       </c>
-      <c r="B1020">
-        <v>51916183000120</v>
+      <c r="B1020" t="s">
+        <v>2140</v>
       </c>
       <c r="C1020" t="s">
         <v>2040</v>
@@ -35656,15 +36418,18 @@
         <v>8</v>
       </c>
       <c r="H1020" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1021" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I1020" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1021" s="1">
         <v>46101</v>
       </c>
-      <c r="B1021">
-        <v>9425553000160</v>
+      <c r="B1021" t="s">
+        <v>2141</v>
       </c>
       <c r="C1021" t="s">
         <v>2041</v>
@@ -35684,8 +36449,11 @@
       <c r="H1021" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1022" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1021">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1022" s="1">
         <v>46102</v>
       </c>
@@ -35708,10 +36476,13 @@
         <v>8</v>
       </c>
       <c r="H1022" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1023" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I1022">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1023" s="1">
         <v>46102</v>
       </c>
@@ -35736,8 +36507,11 @@
       <c r="H1023" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1024" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1023">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1024" s="1">
         <v>46102</v>
       </c>
@@ -35762,8 +36536,11 @@
       <c r="H1024" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="1025" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1024">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1025" s="1">
         <v>46102</v>
       </c>
@@ -35786,10 +36563,13 @@
         <v>8</v>
       </c>
       <c r="H1025" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1026" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I1025">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1026" s="1">
         <v>46102</v>
       </c>
@@ -35812,10 +36592,13 @@
         <v>8</v>
       </c>
       <c r="H1026" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1027" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I1026" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1027" s="1">
         <v>46102</v>
       </c>
@@ -35838,10 +36621,13 @@
         <v>8</v>
       </c>
       <c r="H1027" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1028" spans="1:8" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="I1027" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1028" s="1">
         <v>46102</v>
       </c>
@@ -35864,10 +36650,13 @@
         <v>8</v>
       </c>
       <c r="H1028" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1029" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1028">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1029" s="1">
         <v>46102</v>
       </c>
@@ -35892,8 +36681,11 @@
       <c r="H1029" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1030" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1029">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1030" s="1">
         <v>46102</v>
       </c>
@@ -35916,10 +36708,13 @@
         <v>929</v>
       </c>
       <c r="H1030" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1031" spans="1:8" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="I1030">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1031" s="1">
         <v>46102</v>
       </c>
@@ -35944,8 +36739,11 @@
       <c r="H1031" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1032" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1031">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1032" s="1">
         <v>46102</v>
       </c>
@@ -35968,10 +36766,13 @@
         <v>7</v>
       </c>
       <c r="H1032" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1033" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I1032">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1033" s="1">
         <v>46102</v>
       </c>
@@ -35996,8 +36797,11 @@
       <c r="H1033" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="1034" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1033">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1034" s="1">
         <v>46102</v>
       </c>
@@ -36022,8 +36826,11 @@
       <c r="H1034" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1035" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1034">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1035" s="1">
         <v>46102</v>
       </c>
@@ -36046,10 +36853,13 @@
         <v>8</v>
       </c>
       <c r="H1035" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1036" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="I1035">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1036" s="1">
         <v>46102</v>
       </c>
@@ -36072,10 +36882,13 @@
         <v>8</v>
       </c>
       <c r="H1036" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1037" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1036">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1037" s="1">
         <v>46102</v>
       </c>
@@ -36098,10 +36911,13 @@
         <v>8</v>
       </c>
       <c r="H1037" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1038" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1037">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1038" s="1">
         <v>46102</v>
       </c>
@@ -36126,8 +36942,11 @@
       <c r="H1038" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1039" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1038">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1039" s="1">
         <v>46102</v>
       </c>
@@ -36150,10 +36969,13 @@
         <v>8</v>
       </c>
       <c r="H1039" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="1040" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I1039">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1040" s="1">
         <v>46102</v>
       </c>
@@ -36178,8 +37000,11 @@
       <c r="H1040" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1041" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1040">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1041" s="1">
         <v>46102</v>
       </c>
@@ -36203,6 +37028,1653 @@
       </c>
       <c r="H1041" t="s">
         <v>19</v>
+      </c>
+      <c r="I1041">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1042" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1042" t="s">
+        <v>2142</v>
+      </c>
+      <c r="C1042" t="s">
+        <v>2143</v>
+      </c>
+      <c r="D1042" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1042" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1042" t="s">
+        <v>2144</v>
+      </c>
+      <c r="G1042" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1042" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1042">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1043" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1043" t="s">
+        <v>2145</v>
+      </c>
+      <c r="C1043" t="s">
+        <v>2146</v>
+      </c>
+      <c r="D1043" t="s">
+        <v>1057</v>
+      </c>
+      <c r="F1043" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1043" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1043" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1043">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1044" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1044" t="s">
+        <v>2147</v>
+      </c>
+      <c r="C1044" t="s">
+        <v>2148</v>
+      </c>
+      <c r="D1044" t="s">
+        <v>1057</v>
+      </c>
+      <c r="F1044" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1044" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1044" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1044">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1045" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1045" t="s">
+        <v>2149</v>
+      </c>
+      <c r="C1045" t="s">
+        <v>2150</v>
+      </c>
+      <c r="D1045" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1045" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1045" t="s">
+        <v>1893</v>
+      </c>
+      <c r="G1045" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1045" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1045">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1046" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1046" t="s">
+        <v>2151</v>
+      </c>
+      <c r="C1046" t="s">
+        <v>2152</v>
+      </c>
+      <c r="D1046" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1046" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1046" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1046" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1046" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1047" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1047" t="s">
+        <v>2153</v>
+      </c>
+      <c r="C1047" t="s">
+        <v>2154</v>
+      </c>
+      <c r="D1047" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1047" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1047" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1047" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1047" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1048" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1048" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C1048" t="s">
+        <v>2156</v>
+      </c>
+      <c r="D1048" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1048" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1048" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1048" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1048" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1049" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1049" t="s">
+        <v>2157</v>
+      </c>
+      <c r="C1049" t="s">
+        <v>2158</v>
+      </c>
+      <c r="D1049" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1049" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1049" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1049" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1049" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1050" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1050" t="s">
+        <v>2159</v>
+      </c>
+      <c r="C1050" t="s">
+        <v>2160</v>
+      </c>
+      <c r="D1050" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1050" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1050" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1050" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1050" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1051" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1051" t="s">
+        <v>2161</v>
+      </c>
+      <c r="C1051" t="s">
+        <v>2162</v>
+      </c>
+      <c r="D1051" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1051" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1051" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1051" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1051" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1052" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1052" t="s">
+        <v>2163</v>
+      </c>
+      <c r="C1052" t="s">
+        <v>2164</v>
+      </c>
+      <c r="D1052" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1052" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1052" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1052" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1052" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1053" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1053" t="s">
+        <v>2165</v>
+      </c>
+      <c r="C1053" t="s">
+        <v>2166</v>
+      </c>
+      <c r="D1053" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1053" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1053" t="s">
+        <v>2010</v>
+      </c>
+      <c r="G1053" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1053" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1054" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1054" t="s">
+        <v>2167</v>
+      </c>
+      <c r="C1054" t="s">
+        <v>2168</v>
+      </c>
+      <c r="D1054" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1054" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1054" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1054" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1054" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1055" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1055" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C1055" t="s">
+        <v>2170</v>
+      </c>
+      <c r="D1055" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1055" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1055" t="s">
+        <v>2010</v>
+      </c>
+      <c r="G1055" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1055" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1056" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1056" t="s">
+        <v>2171</v>
+      </c>
+      <c r="C1056" t="s">
+        <v>2172</v>
+      </c>
+      <c r="D1056" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1056" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1056" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1056" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1056" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1057" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1057" t="s">
+        <v>2173</v>
+      </c>
+      <c r="C1057" t="s">
+        <v>2174</v>
+      </c>
+      <c r="D1057" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1057" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1057" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1057" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1057" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1058" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1058" t="s">
+        <v>2175</v>
+      </c>
+      <c r="C1058" t="s">
+        <v>2176</v>
+      </c>
+      <c r="D1058" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1058" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1058" t="s">
+        <v>2010</v>
+      </c>
+      <c r="G1058" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1058" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1059" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1059" t="s">
+        <v>2177</v>
+      </c>
+      <c r="C1059" t="s">
+        <v>2178</v>
+      </c>
+      <c r="D1059" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1059" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1059" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1059" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1059" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1060" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1060" t="s">
+        <v>2179</v>
+      </c>
+      <c r="C1060" t="s">
+        <v>2180</v>
+      </c>
+      <c r="D1060" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1060" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1060" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1060" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1060" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1061" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1061" t="s">
+        <v>2181</v>
+      </c>
+      <c r="C1061" t="s">
+        <v>2182</v>
+      </c>
+      <c r="D1061" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1061" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1061" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1061" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1061" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1062" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1062" t="s">
+        <v>2183</v>
+      </c>
+      <c r="C1062" t="s">
+        <v>2184</v>
+      </c>
+      <c r="D1062" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1062" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1062" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1062" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1062" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1063" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1063" t="s">
+        <v>2185</v>
+      </c>
+      <c r="C1063" t="s">
+        <v>2186</v>
+      </c>
+      <c r="D1063" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1063" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1063" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1063" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1063" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1064" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1064" t="s">
+        <v>2187</v>
+      </c>
+      <c r="C1064" t="s">
+        <v>2188</v>
+      </c>
+      <c r="D1064" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1064" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1064" t="s">
+        <v>1893</v>
+      </c>
+      <c r="G1064" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1064" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1065" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1065" t="s">
+        <v>2189</v>
+      </c>
+      <c r="C1065" t="s">
+        <v>2190</v>
+      </c>
+      <c r="D1065" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1065" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1065" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1065" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1065" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1066" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1066" t="s">
+        <v>2191</v>
+      </c>
+      <c r="C1066" t="s">
+        <v>2192</v>
+      </c>
+      <c r="D1066" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1066" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1066" t="s">
+        <v>1753</v>
+      </c>
+      <c r="G1066" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1066" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1067" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1067" t="s">
+        <v>2193</v>
+      </c>
+      <c r="C1067" t="s">
+        <v>2194</v>
+      </c>
+      <c r="D1067" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1067" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1067" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1067" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1067" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1068" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1068" t="s">
+        <v>2195</v>
+      </c>
+      <c r="C1068" t="s">
+        <v>2196</v>
+      </c>
+      <c r="D1068" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1068" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1068" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1068" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1068" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1069" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1069" t="s">
+        <v>2197</v>
+      </c>
+      <c r="C1069" t="s">
+        <v>2198</v>
+      </c>
+      <c r="D1069" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1069" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1069" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1069" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1069" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1070" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1070" t="s">
+        <v>2199</v>
+      </c>
+      <c r="C1070" t="s">
+        <v>2200</v>
+      </c>
+      <c r="D1070" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1070" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1070" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1070" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1070" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1071" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1071" t="s">
+        <v>2201</v>
+      </c>
+      <c r="C1071" t="s">
+        <v>2202</v>
+      </c>
+      <c r="D1071" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1071" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1071" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1071" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1071" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1072" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1072" t="s">
+        <v>2203</v>
+      </c>
+      <c r="C1072" t="s">
+        <v>2204</v>
+      </c>
+      <c r="D1072" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1072" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1072" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1072" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1072" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1073" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1073" t="s">
+        <v>2205</v>
+      </c>
+      <c r="C1073" t="s">
+        <v>2206</v>
+      </c>
+      <c r="D1073" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1073" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1073" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1073" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1073" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1074" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1074" t="s">
+        <v>2207</v>
+      </c>
+      <c r="C1074" t="s">
+        <v>2208</v>
+      </c>
+      <c r="D1074" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1074" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1074" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1074" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1074" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1075" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1075" t="s">
+        <v>2209</v>
+      </c>
+      <c r="C1075" t="s">
+        <v>2210</v>
+      </c>
+      <c r="D1075" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1075" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1075" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1075" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1075" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1076" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1076" t="s">
+        <v>2211</v>
+      </c>
+      <c r="C1076" t="s">
+        <v>2212</v>
+      </c>
+      <c r="D1076" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1076" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1076" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1076" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1076" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1077" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1077" t="s">
+        <v>2213</v>
+      </c>
+      <c r="C1077" t="s">
+        <v>2214</v>
+      </c>
+      <c r="D1077" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1077" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1077" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1077" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1077" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1078" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1078" t="s">
+        <v>2215</v>
+      </c>
+      <c r="C1078" t="s">
+        <v>2216</v>
+      </c>
+      <c r="D1078" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1078" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1078" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1078" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1078" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1079" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1079" t="s">
+        <v>2217</v>
+      </c>
+      <c r="C1079" t="s">
+        <v>2218</v>
+      </c>
+      <c r="D1079" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1079" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1079" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1079" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1079" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1080" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1080" t="s">
+        <v>2219</v>
+      </c>
+      <c r="C1080" t="s">
+        <v>2220</v>
+      </c>
+      <c r="D1080" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1080" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1080" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1080" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1080" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1081" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1081" t="s">
+        <v>2221</v>
+      </c>
+      <c r="C1081" t="s">
+        <v>2222</v>
+      </c>
+      <c r="D1081" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1081" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1081" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1081" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1081" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1082" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1082" t="s">
+        <v>2223</v>
+      </c>
+      <c r="C1082" t="s">
+        <v>2224</v>
+      </c>
+      <c r="D1082" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1082" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1082" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1082" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1082" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1083" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1083" t="s">
+        <v>2225</v>
+      </c>
+      <c r="C1083" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D1083" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1083" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1083" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1083" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1083" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1084" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1084" t="s">
+        <v>2227</v>
+      </c>
+      <c r="C1084" t="s">
+        <v>2228</v>
+      </c>
+      <c r="D1084" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1084" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1084" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1084" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1084" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1085" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1085" t="s">
+        <v>2229</v>
+      </c>
+      <c r="C1085" t="s">
+        <v>2230</v>
+      </c>
+      <c r="D1085" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1085" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1085" t="s">
+        <v>2010</v>
+      </c>
+      <c r="G1085" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1085" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1086" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1086" t="s">
+        <v>2231</v>
+      </c>
+      <c r="C1086" t="s">
+        <v>2232</v>
+      </c>
+      <c r="D1086" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1086" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1086" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1086" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1086" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1087" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1087" t="s">
+        <v>2233</v>
+      </c>
+      <c r="C1087" t="s">
+        <v>2234</v>
+      </c>
+      <c r="D1087" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1087" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1087" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1087" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1087" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1088" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1088" t="s">
+        <v>2235</v>
+      </c>
+      <c r="C1088" t="s">
+        <v>2236</v>
+      </c>
+      <c r="D1088" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1088" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1088" t="s">
+        <v>2237</v>
+      </c>
+      <c r="G1088" t="s">
+        <v>929</v>
+      </c>
+      <c r="H1088" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1089" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1089" t="s">
+        <v>2238</v>
+      </c>
+      <c r="C1089" t="s">
+        <v>2239</v>
+      </c>
+      <c r="D1089" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1089" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1089" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1089" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1089" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1090" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1090" t="s">
+        <v>2240</v>
+      </c>
+      <c r="C1090" t="s">
+        <v>2241</v>
+      </c>
+      <c r="D1090" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1090" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1090" t="s">
+        <v>1893</v>
+      </c>
+      <c r="G1090" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1090" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1091" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1091" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C1091" t="s">
+        <v>2243</v>
+      </c>
+      <c r="D1091" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1091" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1091" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1091" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1091" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1092" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1092" t="s">
+        <v>2244</v>
+      </c>
+      <c r="C1092" t="s">
+        <v>2245</v>
+      </c>
+      <c r="D1092" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1092" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1092" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1092" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1092" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1093" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1093" t="s">
+        <v>2246</v>
+      </c>
+      <c r="C1093" t="s">
+        <v>2247</v>
+      </c>
+      <c r="D1093" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1093" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1093" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1093" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1093" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1094" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1094" t="s">
+        <v>2248</v>
+      </c>
+      <c r="C1094" t="s">
+        <v>2249</v>
+      </c>
+      <c r="D1094" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1094" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1094" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1094" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1095" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1095" t="s">
+        <v>2250</v>
+      </c>
+      <c r="C1095" t="s">
+        <v>2251</v>
+      </c>
+      <c r="D1095" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1095" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1095" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1095" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1095" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1096" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1096" t="s">
+        <v>2252</v>
+      </c>
+      <c r="C1096" t="s">
+        <v>2253</v>
+      </c>
+      <c r="D1096" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1096" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1096" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1096" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1096" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1097" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1097" t="s">
+        <v>2254</v>
+      </c>
+      <c r="C1097" t="s">
+        <v>2255</v>
+      </c>
+      <c r="D1097" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1097" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1097" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1097" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1097" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1098" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1098" t="s">
+        <v>2256</v>
+      </c>
+      <c r="C1098" t="s">
+        <v>2257</v>
+      </c>
+      <c r="D1098" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E1098" t="s">
+        <v>1241</v>
+      </c>
+      <c r="F1098" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1098" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1098" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1099" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1099" t="s">
+        <v>2258</v>
+      </c>
+      <c r="C1099" t="s">
+        <v>2259</v>
+      </c>
+      <c r="D1099" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1099" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1099" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1099" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1099" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1100" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1100" t="s">
+        <v>2260</v>
+      </c>
+      <c r="C1100" t="s">
+        <v>2261</v>
+      </c>
+      <c r="D1100" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1100" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1100" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1100" t="s">
+        <v>2262</v>
+      </c>
+      <c r="H1100" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1101" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1101" t="s">
+        <v>2263</v>
+      </c>
+      <c r="C1101" t="s">
+        <v>2264</v>
+      </c>
+      <c r="D1101" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1101" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1101" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1101" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1101" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1102" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1102" t="s">
+        <v>2265</v>
+      </c>
+      <c r="C1102" t="s">
+        <v>2266</v>
+      </c>
+      <c r="D1102" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1102" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1102" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1102" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1102" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1103" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1103" t="s">
+        <v>2267</v>
+      </c>
+      <c r="C1103" t="s">
+        <v>2268</v>
+      </c>
+      <c r="D1103" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E1103" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1103" t="s">
+        <v>1753</v>
+      </c>
+      <c r="G1103" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1103" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1104" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B1104" t="s">
+        <v>2269</v>
+      </c>
+      <c r="C1104" t="s">
+        <v>2270</v>
+      </c>
+      <c r="D1104" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E1104" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F1104" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1104" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1104" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>